<commit_message>
Excel parity: add Developer Project Finance workbook (5th model)
Generated newman-projectfinance-model.xlsx (gearing/DSCR/project+equity IRR via
live IRR formulas); added to combined pack (now 6 sheets); models.html updated to
5 models + new download card.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/newman-energy-models.xlsx
+++ b/models/newman-energy-models.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Savings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exit NPV-DCF" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BESS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project finance" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="169" formatCode="0.0"/>
     <numFmt numFmtId="170" formatCode="0.0&quot; yrs&quot;"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,6 +95,10 @@
       <color rgb="005F5870"/>
       <sz val="9"/>
     </font>
+    <font>
+      <color rgb="005F5870"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -144,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -207,6 +212,10 @@
     <xf numFmtId="170" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -572,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -634,17 +643,24 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5. Developer Project Finance — gearing, DSCR and levered equity IRR</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>These mirror the interactive calculators on the Academy site exactly.</t>
-        </is>
-      </c>
+      <c r="A12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>These mirror the interactive calculators on the Academy site exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>All figures are illustrative defaults for Europe / Czechia. Not investment advice.</t>
         </is>
@@ -3100,4 +3116,686 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Developer Project Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Gearing, DSCR &amp; levered equity IRR  ·  Newman Energy Academy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="8" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Capex</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Equity IRR (levered)</t>
+        </is>
+      </c>
+      <c r="F5" s="30">
+        <f>IFERROR(IRR(J12:J47),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Annual net cash flow (CFADS)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>EUR / yr</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Project IRR (unlevered)</t>
+        </is>
+      </c>
+      <c r="F6" s="15">
+        <f>IFERROR(IRR(I12:I47),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Debt share (gearing)</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>DSCR (year 1)</t>
+        </is>
+      </c>
+      <c r="F7" s="26">
+        <f>$B$6/$F$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Loan interest rate</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Equity required</t>
+        </is>
+      </c>
+      <c r="F8" s="24">
+        <f>$B$5*(1-$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Loan tenor</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Annual debt service</t>
+        </is>
+      </c>
+      <c r="F9" s="24">
+        <f>$B$5*$B$7*$B$8/(1-(1+$B$8)^-$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Asset life</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Equity payback (approx)</t>
+        </is>
+      </c>
+      <c r="F10" s="29">
+        <f>IF(($B$6-$F$9)&gt;0,$F$8/($B$6-$F$9),"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="H11" s="31" t="inlineStr">
+        <is>
+          <t>yr</t>
+        </is>
+      </c>
+      <c r="I11" s="31" t="inlineStr">
+        <is>
+          <t>proj CF</t>
+        </is>
+      </c>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>equity CF</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Inputs are blue; results recalc. Debt sized at level annual service.</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="22">
+        <f>-$B$5</f>
+        <v/>
+      </c>
+      <c r="J12" s="22">
+        <f>-$F$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="22">
+        <f>IF(1&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J13" s="22">
+        <f>IF(1&lt;=$B$10,IF(1&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="22">
+        <f>IF(2&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J14" s="22">
+        <f>IF(2&lt;=$B$10,IF(2&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="22">
+        <f>IF(3&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J15" s="22">
+        <f>IF(3&lt;=$B$10,IF(3&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" s="22">
+        <f>IF(4&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J16" s="22">
+        <f>IF(4&lt;=$B$10,IF(4&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="H17" t="n">
+        <v>5</v>
+      </c>
+      <c r="I17" s="22">
+        <f>IF(5&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J17" s="22">
+        <f>IF(5&lt;=$B$10,IF(5&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="H18" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="22">
+        <f>IF(6&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J18" s="22">
+        <f>IF(6&lt;=$B$10,IF(6&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="H19" t="n">
+        <v>7</v>
+      </c>
+      <c r="I19" s="22">
+        <f>IF(7&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J19" s="22">
+        <f>IF(7&lt;=$B$10,IF(7&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="H20" t="n">
+        <v>8</v>
+      </c>
+      <c r="I20" s="22">
+        <f>IF(8&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J20" s="22">
+        <f>IF(8&lt;=$B$10,IF(8&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="H21" t="n">
+        <v>9</v>
+      </c>
+      <c r="I21" s="22">
+        <f>IF(9&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J21" s="22">
+        <f>IF(9&lt;=$B$10,IF(9&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="H22" t="n">
+        <v>10</v>
+      </c>
+      <c r="I22" s="22">
+        <f>IF(10&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J22" s="22">
+        <f>IF(10&lt;=$B$10,IF(10&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="H23" t="n">
+        <v>11</v>
+      </c>
+      <c r="I23" s="22">
+        <f>IF(11&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J23" s="22">
+        <f>IF(11&lt;=$B$10,IF(11&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="H24" t="n">
+        <v>12</v>
+      </c>
+      <c r="I24" s="22">
+        <f>IF(12&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J24" s="22">
+        <f>IF(12&lt;=$B$10,IF(12&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="H25" t="n">
+        <v>13</v>
+      </c>
+      <c r="I25" s="22">
+        <f>IF(13&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J25" s="22">
+        <f>IF(13&lt;=$B$10,IF(13&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="H26" t="n">
+        <v>14</v>
+      </c>
+      <c r="I26" s="22">
+        <f>IF(14&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J26" s="22">
+        <f>IF(14&lt;=$B$10,IF(14&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="H27" t="n">
+        <v>15</v>
+      </c>
+      <c r="I27" s="22">
+        <f>IF(15&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J27" s="22">
+        <f>IF(15&lt;=$B$10,IF(15&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="H28" t="n">
+        <v>16</v>
+      </c>
+      <c r="I28" s="22">
+        <f>IF(16&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J28" s="22">
+        <f>IF(16&lt;=$B$10,IF(16&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="H29" t="n">
+        <v>17</v>
+      </c>
+      <c r="I29" s="22">
+        <f>IF(17&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J29" s="22">
+        <f>IF(17&lt;=$B$10,IF(17&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="H30" t="n">
+        <v>18</v>
+      </c>
+      <c r="I30" s="22">
+        <f>IF(18&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J30" s="22">
+        <f>IF(18&lt;=$B$10,IF(18&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="H31" t="n">
+        <v>19</v>
+      </c>
+      <c r="I31" s="22">
+        <f>IF(19&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J31" s="22">
+        <f>IF(19&lt;=$B$10,IF(19&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="H32" t="n">
+        <v>20</v>
+      </c>
+      <c r="I32" s="22">
+        <f>IF(20&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J32" s="22">
+        <f>IF(20&lt;=$B$10,IF(20&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="H33" t="n">
+        <v>21</v>
+      </c>
+      <c r="I33" s="22">
+        <f>IF(21&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J33" s="22">
+        <f>IF(21&lt;=$B$10,IF(21&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="H34" t="n">
+        <v>22</v>
+      </c>
+      <c r="I34" s="22">
+        <f>IF(22&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J34" s="22">
+        <f>IF(22&lt;=$B$10,IF(22&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="H35" t="n">
+        <v>23</v>
+      </c>
+      <c r="I35" s="22">
+        <f>IF(23&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J35" s="22">
+        <f>IF(23&lt;=$B$10,IF(23&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="H36" t="n">
+        <v>24</v>
+      </c>
+      <c r="I36" s="22">
+        <f>IF(24&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J36" s="22">
+        <f>IF(24&lt;=$B$10,IF(24&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="H37" t="n">
+        <v>25</v>
+      </c>
+      <c r="I37" s="22">
+        <f>IF(25&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J37" s="22">
+        <f>IF(25&lt;=$B$10,IF(25&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="H38" t="n">
+        <v>26</v>
+      </c>
+      <c r="I38" s="22">
+        <f>IF(26&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J38" s="22">
+        <f>IF(26&lt;=$B$10,IF(26&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="H39" t="n">
+        <v>27</v>
+      </c>
+      <c r="I39" s="22">
+        <f>IF(27&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J39" s="22">
+        <f>IF(27&lt;=$B$10,IF(27&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="H40" t="n">
+        <v>28</v>
+      </c>
+      <c r="I40" s="22">
+        <f>IF(28&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J40" s="22">
+        <f>IF(28&lt;=$B$10,IF(28&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="H41" t="n">
+        <v>29</v>
+      </c>
+      <c r="I41" s="22">
+        <f>IF(29&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J41" s="22">
+        <f>IF(29&lt;=$B$10,IF(29&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="H42" t="n">
+        <v>30</v>
+      </c>
+      <c r="I42" s="22">
+        <f>IF(30&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J42" s="22">
+        <f>IF(30&lt;=$B$10,IF(30&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43" t="n">
+        <v>31</v>
+      </c>
+      <c r="I43" s="22">
+        <f>IF(31&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J43" s="22">
+        <f>IF(31&lt;=$B$10,IF(31&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="H44" t="n">
+        <v>32</v>
+      </c>
+      <c r="I44" s="22">
+        <f>IF(32&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J44" s="22">
+        <f>IF(32&lt;=$B$10,IF(32&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="H45" t="n">
+        <v>33</v>
+      </c>
+      <c r="I45" s="22">
+        <f>IF(33&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J45" s="22">
+        <f>IF(33&lt;=$B$10,IF(33&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="H46" t="n">
+        <v>34</v>
+      </c>
+      <c r="I46" s="22">
+        <f>IF(34&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J46" s="22">
+        <f>IF(34&lt;=$B$10,IF(34&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="H47" t="n">
+        <v>35</v>
+      </c>
+      <c r="I47" s="22">
+        <f>IF(35&lt;=$B$10,$B$6,0)</f>
+        <v/>
+      </c>
+      <c r="J47" s="22">
+        <f>IF(35&lt;=$B$10,IF(35&lt;=$B$9,$B$6-$F$9,$B$6),0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>